<commit_message>
Clarify no-match venues report shows all rows
</commit_message>
<xml_diff>
--- a/reports/openalex_only_venues_no_crossref_journal_match.xlsx
+++ b/reports/openalex_only_venues_no_crossref_journal_match.xlsx
@@ -9,7 +9,7 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="No_Crossref_Journal_Match" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Top_No_Match_Compact" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="All_No_Match_Compact" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -511,11 +511,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D17"/>
+  <dimension ref="A1:D19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
-    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="55" customWidth="1" min="2" max="2"/>
     <col width="24" customWidth="1" min="3" max="3"/>
     <col width="24" customWidth="1" min="4" max="4"/>
   </cols>
@@ -530,7 +530,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Subset of OpenAlex-only venues from the current collected dataset where Crossref journal lookup did not find a journal match.</t>
+          <t>Complete subset of OpenAlex-only venues from the current collected dataset where Crossref journal lookup did not find a journal match.</t>
         </is>
       </c>
     </row>
@@ -591,7 +591,7 @@
     <row r="12">
       <c r="A12" s="5" t="inlineStr">
         <is>
-          <t>These venues were observed only through OpenAlex in this project dataset and were not matched to a Crossref journal title in the follow-up lookup. This often indicates repositories, preprint platforms, institutional sources, conference/proceeding records, or noisy/non-journal source names rather than reputable manufacturing journals.</t>
+          <t>These are all venues observed only through OpenAlex in this project dataset and not matched to a Crossref journal title in the follow-up lookup. This often indicates repositories, preprint platforms, institutional sources, conference/proceeding records, or noisy/non-journal source names rather than reputable manufacturing journals.</t>
         </is>
       </c>
     </row>
@@ -618,6 +618,18 @@
       <c r="B17" t="inlineStr">
         <is>
           <t>2026-06-17 12:02:01 KST</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>Sheet note</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>All_No_Match_Compact contains all 93 no-match venues, not a top-N sample.</t>
         </is>
       </c>
     </row>

</xml_diff>